<commit_message>
Barvy podle MicroStationu, vyhledávání a poznámky u chyb, opravy
- čísla barev v pravidlech jsou výchozí čísla MicroStationu, porovnání podle RGB;
  načtení vlastní barevné tabulky (color.tbl nebo text), hlášení barvy jako čísla MS
- tloušťky MicroStationu (wt) se nehlásí jako chyba, jen poznámka
- vzorový výkres navrhuje barvy v číslech MicroStationu
- vyhledávání v seznamu chyb, poznámka k chybě, naposledy otevřené výkresy
- oprava: podklad pod výkresem po načtení jiného výkresu, porovnání při
  opakované kontrole počítá i shodné chyby
- CI testuje přímo sestavené .exe (kontrola, exporty, spuštění okna), TESTOVANI.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018zQVeabg8D28useAA36Kin
</commit_message>
<xml_diff>
--- a/ukazky/tabulka_atributu.xlsx
+++ b/ukazky/tabulka_atributu.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (červená)</t>
+          <t>3 (červená)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (zelená)</t>
+          <t>2 (zelená)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5 (modrá)</t>
+          <t>1 (modrá)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -737,7 +737,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -781,7 +781,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -849,7 +849,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>

</xml_diff>